<commit_message>
created python scripts and updated the html extraction for trane
</commit_message>
<xml_diff>
--- a/trane_news.xlsx
+++ b/trane_news.xlsx
@@ -572,11 +572,11 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>46062.47213317751</v>
+        <v>46062.505836739</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications. Trane® Connect™ is our secure, cloud-based customer portal to access your building systems to remotely monitor and manage building systems, and conduct routine maintenance. Products Services Support Education &amp; Training Industries About North America Latin America Europe Middle East Asia Pacific Press Release Media Contact Trane Technologies Media Relations Trane by Trane Technologies Quick Facts DAVIDSON, N.C., Feb. 2, 2026 – Trane® – by Trane Technologies (NYSE: TT), a global climate innovator, today announced the launch of Trane Cloud, a digital hub designed to transform how building operators, facility teams, and energy managers interact with their buildings. Trane Cloud brings together analytics, applications and services into one secure, seamless digital experience, empowering teams to operate buildings more efficiently, reliably and sustainably. For years, building professionals have navigated a complex web of systems, with valuable data often trapped in proprietary interfaces or fragmented dashboards. Trane Cloud addresses this challenge by creating a single, intelligent data foundation that provides portfolio- and site-level visibility, delivering actionable insights for energy optimization and prioritized recommendations to streamline operations and enhance decision-making. “In today’s increasingly digital world, building operators are flooded with data from their buildings and need a way to make sense of it all,” said Riaz Raihan, Senior Vice President and Chief Digital Officer of Trane Technologies. “Trane Cloud is our answer. It serves as the entry point for the digital experience, revolutionizing building operations by bringing everything together in one place to optimize performance. Trane Cloud is the foundation for a smarter, more efficient building, helping our customers meet their goals for sustainability, efficiency, reliability and comfort.” Trane Cloud delivers a powerful suite of Trane applications and digital services to help building teams manage and prioritize their work more effectively. Key benefits of Trane Cloud include: Trane Cloud is designed for a wide range of customers, including facility teams focused on efficient operations; building teams focused on long-term performance; energy managers aiming to reduce carbon emissions; and organizations of all sizes seeking consistent, data-driven oversight across their portfolios. By providing a secure, scalable, and intuitive platform, Trane is empowering customers to unlock the full potential of their buildings. About Trane Trane – by Trane Technologies (NYSE: TT), a global climate innovator – creates comfortable, energy efficient indoor environments for commercial and residential applications. For more information, please visit www.trane.com or www.tranetechnologies.com.</t>
+          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications. Trane® Connect™ is our secure, cloud-based customer portal to access your building systems to remotely monitor and manage building systems, and conduct routine maintenance. Products Services Support Education &amp; Training Industries About North America Latin America Europe Middle East Asia Pacific Press Release Media Contact Trane Technologies Media Relations Trane by Trane Technologies Quick Facts DAVIDSON, N.C., Feb. 2, 2026 – Trane® – by Trane Technologies (NYSE: TT), a global climate innovator, today announced the launch of Trane Cloud, a digital hub designed to transform how building operators, facility teams, and energy managers interact with their buildings. Trane Cloud brings together analytics, applications and services into one secure, seamless digital experience, empowering teams to operate buildings more efficiently, reliably and sustainably. For years, building professionals have navigated a complex web of systems, with valuable data often trapped in proprietary interfaces or fragmented dashboards. Trane Cloud addresses this challenge by creating a single, intelligent data foundation that provides portfolio- and site-level visibility, delivering actionable insights for energy optimization and prioritized recommendations to streamline operations and enhance decision-making. “In today’s increasingly digital world, building operators are flooded with data from their buildings and need a way to make sense of it all,” said Riaz Raihan, Senior Vice President and Chief Digital Officer of Trane Technologies. “Trane Cloud is our answer. It serves as the entry point for the digital experience, revolutionizing building operations by bringing everything together in one place to optimize performance. Trane Cloud is the foundation for a smarter, more efficient building, helping our customers meet their goals for sustainability, efficiency, reliability and comfort.” Trane Cloud delivers a powerful suite of Trane applications and digital services to help building teams manage and prioritize their work more effectively. Key benefits of Trane Cloud include: Trane Cloud is designed for a wide range of customers, including facility teams focused on efficient operations; building teams focused on long-term performance; energy managers aiming to reduce carbon emissions; and organizations of all sizes seeking consistent, data-driven oversight across their portfolios. By providing a secure, scalable, and intuitive platform, Trane is empowering customers to unlock the full potential of their buildings.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -602,11 +602,11 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>46062.47213820922</v>
+        <v>46062.50584230535</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications. Trane® Connect™ is our secure, cloud-based customer portal to access your building systems to remotely monitor and manage building systems, and conduct routine maintenance. Products Services Support Education &amp; Training Industries About North America Latin America Europe Middle East Asia Pacific Press Release Garrett Motion’s breakthrough oil-free centrifugal compressor technology exclusively available through Trane portfolio for commercial applications. Media Contact Trane Technologies Media Relations Trane by Trane Technologies Quick Facts DAVIDSON, N.C., PLYMOUTH, MI, and ROLLE, Switzerland, Feb. 2, 2026 – Trane® – by Trane Technologies (NYSE: TT), a global climate innovator, and Garrett Motion (Nasdaq: GTX), a global leader in differentiated turbocharging and electrification technologies, today announced a strategic collaboration to accelerate next generation, oil-free centrifugal compressor technology for commercial heating, ventilation and air conditioning (HVAC) applications. The collaboration brings together Trane’s industry-leading Commercial HVAC system expertise and performance with Garrett’s breakthrough oil-free high-speed centrifugal compressor technology, which has already demonstrated clear performance benefits including major energy efficiency gains in Trane’s testing. Together, Trane and Garrett will launch the next generation of high efficiency HVAC systems and accelerate the adoption of ultra-low global warming potential refrigerants. The companies will jointly develop and integrate advanced compressor solutions across a broad portfolio of Trane systems, including unitary rooftop units, modular chillers, and large capacity chillers for a variety of applications. Field testing and production of the jointly developed technology are scheduled to begin in 2026, marking a major milestone in the companies’ shared focus on innovation, energy efficiency and lower environmental impact. “This collaboration advances our commitment to lead the industry with high-performing, energy efficient solutions that support our customers’ decarbonization goals,” said Mauro Atalla, Chief Technology and Sustainability Officer, Trane Technologies. “Garrett Motion brings deep expertise and a shared commitment to quality with their oil-free centrifugal compressor technology. Together, we are accelerating innovation that will shape the next era of sustainable HVAC systems.” The collaboration establishes a framework for shared engineering, design and field testing activities across global markets. It also includes joint exploration of future applications, including high-speed centrifugal technologies for smaller capacity HVAC systems, distributed cooling and other emerging cooling needs. “Garrett is proud to partner with Trane Technologies, one of the most respected names in the HVAC industry, as we expand the use of our unique oil-free high-speed compressor technology in the industrial space,” said Olivier Rabiller, President and CEO of Garrett Motion. “Combining this technology proven in several automotive applications with Trane’s system-level leadership enables customers to benefit from a better, more energy-efficient and cost-effective HVAC system while advancing their sustainability goals.” The collaboration reinforces both organizations’ commitment to industry-leading performance, reliability and customer value. About Trane Trane – by Trane Technologies (NYSE: TT), a global climate innovator – creates comfortable, energy efficient indoor environments for commercial and residential applications. For more information, please visit www.trane.com or www.tranetechnologies.com.</t>
+          <t>Selecting a language changes the language and content on the Trane site. Trane ComfortSite is an extranet site designed to save you time. With your secure login, you can: This is the login for Trane® Connect™ and other Trane® commercial applications. Trane® Connect™ is our secure, cloud-based customer portal to access your building systems to remotely monitor and manage building systems, and conduct routine maintenance. Products Services Support Education &amp; Training Industries About North America Latin America Europe Middle East Asia Pacific Press Release Garrett Motion’s breakthrough oil-free centrifugal compressor technology exclusively available through Trane portfolio for commercial applications. Media Contact Trane Technologies Media Relations Trane by Trane Technologies Quick Facts DAVIDSON, N.C., PLYMOUTH, MI, and ROLLE, Switzerland, Feb. 2, 2026 – Trane® – by Trane Technologies (NYSE: TT), a global climate innovator, and Garrett Motion (Nasdaq: GTX), a global leader in differentiated turbocharging and electrification technologies, today announced a strategic collaboration to accelerate next generation, oil-free centrifugal compressor technology for commercial heating, ventilation and air conditioning (HVAC) applications. The collaboration brings together Trane’s industry-leading Commercial HVAC system expertise and performance with Garrett’s breakthrough oil-free high-speed centrifugal compressor technology, which has already demonstrated clear performance benefits including major energy efficiency gains in Trane’s testing. Together, Trane and Garrett will launch the next generation of high efficiency HVAC systems and accelerate the adoption of ultra-low global warming potential refrigerants. The companies will jointly develop and integrate advanced compressor solutions across a broad portfolio of Trane systems, including unitary rooftop units, modular chillers, and large capacity chillers for a variety of applications. Field testing and production of the jointly developed technology are scheduled to begin in 2026, marking a major milestone in the companies’ shared focus on innovation, energy efficiency and lower environmental impact. “This collaboration advances our commitment to lead the industry with high-performing, energy efficient solutions that support our customers’ decarbonization goals,” said Mauro Atalla, Chief Technology and Sustainability Officer, Trane Technologies. “Garrett Motion brings deep expertise and a shared commitment to quality with their oil-free centrifugal compressor technology. Together, we are accelerating innovation that will shape the next era of sustainable HVAC systems.” The collaboration establishes a framework for shared engineering, design and field testing activities across global markets. It also includes joint exploration of future applications, including high-speed centrifugal technologies for smaller capacity HVAC systems, distributed cooling and other emerging cooling needs. “Garrett is proud to partner with Trane Technologies, one of the most respected names in the HVAC industry, as we expand the use of our unique oil-free high-speed compressor technology in the industrial space,” said Olivier Rabiller, President and CEO of Garrett Motion. “Combining this technology proven in several automotive applications with Trane’s system-level leadership enables customers to benefit from a better, more energy-efficient and cost-effective HVAC system while advancing their sustainability goals.” The collaboration reinforces both organizations’ commitment to industry-leading performance, reliability and customer value.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">

</xml_diff>